<commit_message>
Separadores con dos puntos y comas, y memorias actualizadas
</commit_message>
<xml_diff>
--- a/avionica/comparativa_stm32.xlsx
+++ b/avionica/comparativa_stm32.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/edenrochman/Library/Mobile Documents/com~apple~CloudDocs/Universidad de Valencia/faraday/avionica/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_127C967BA328DCABA6DEA159C714B26127DB4062" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_B6BD58E99FB50310E2081508EDA0C537AA9A4ED4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8200" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,9 +29,6 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -39,10 +36,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="78">
   <si>
-    <t>Comparativa de microcontroladores STM32 · Aviónica de vuelo</t>
-  </si>
-  <si>
-    <t>Ejercicio 1a · Faraday Rocketry UPV</t>
+    <t>Comparativa de microcontroladores STM32: aviónica de vuelo</t>
+  </si>
+  <si>
+    <t>Faraday Rocketry UPV, ejercicio 1a</t>
   </si>
   <si>
     <t>Criterio</t>
@@ -163,10 +160,10 @@
     <t>Fuentes: datasheets de STMicroelectronics DS8626 Rev 12 (STM32F405), DS10314 Rev 8 (STM32F411) y DS12110 Rev 11 (STM32H743). Estimación de carga de CPU en la hoja «Carga CPU».</t>
   </si>
   <si>
-    <t>Estimación de carga de CPU en vuelo · STM32F405</t>
-  </si>
-  <si>
-    <t>Ejercicio 1a · Valores en azul: supuestos de la estimación · En negro: valores calculados</t>
+    <t>Estimación de carga de CPU en vuelo: STM32F405</t>
+  </si>
+  <si>
+    <t>Ejercicio 1a, en azul los supuestos de la estimación y en negro los valores calculados</t>
   </si>
   <si>
     <t>Supuestos</t>
@@ -387,7 +384,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -423,12 +420,117 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -439,84 +541,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -852,274 +876,274 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
     </row>
     <row r="4" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="24"/>
     </row>
     <row r="6" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="3">
         <v>168</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="4">
         <v>100</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="4">
         <v>480</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="24"/>
     </row>
     <row r="10" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="3">
         <v>1024</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="4">
         <v>512</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="4">
         <v>2048</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="3">
         <v>192</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="4">
         <v>128</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="4">
         <v>1056</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="24"/>
     </row>
     <row r="13" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="14">
+      <c r="B13" s="3">
         <v>3</v>
       </c>
-      <c r="C13" s="15">
+      <c r="C13" s="4">
         <v>5</v>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="14">
+      <c r="B14" s="3">
         <v>3</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="4">
         <v>3</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="14">
+      <c r="B17" s="3">
         <v>12</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="4">
         <v>8</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="24"/>
     </row>
     <row r="20" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="4" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="24"/>
     </row>
     <row r="23" spans="1:4" ht="259.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="24"/>
     </row>
     <row r="25" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A25:D25"/>
     <mergeCell ref="A19:D19"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A2:D2"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B23:D23"/>
     <mergeCell ref="A12:D12"/>
+    <mergeCell ref="B22:D22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1143,485 +1167,485 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
     </row>
     <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
     </row>
     <row r="4" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
     </row>
     <row r="5" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="19">
+      <c r="B5" s="8">
         <v>5</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="23"/>
     </row>
     <row r="6" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="20">
+      <c r="B6" s="9">
         <v>20000000</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="31" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
     </row>
     <row r="7" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="10">
         <v>0.3</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
     </row>
     <row r="8" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="20">
+      <c r="B8" s="9">
         <v>100000000</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
     </row>
     <row r="9" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B9" s="20">
+      <c r="B9" s="9">
         <v>168000000</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="23"/>
     </row>
     <row r="10" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="20">
+      <c r="B10" s="9">
         <v>480000000</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
     </row>
     <row r="12" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
     </row>
     <row r="13" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="22" t="s">
+      <c r="D13" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="E13" s="22" t="s">
+      <c r="E13" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="F13" s="22" t="s">
+      <c r="F13" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="G13" s="22" t="s">
+      <c r="G13" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="H13" s="22" t="s">
+      <c r="H13" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="I13" s="22" t="s">
+      <c r="I13" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="J13" s="22" t="s">
+      <c r="J13" s="11" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="23">
+      <c r="B14" s="12">
         <v>3</v>
       </c>
-      <c r="C14" s="23">
+      <c r="C14" s="12">
         <v>2</v>
       </c>
-      <c r="D14" s="20">
+      <c r="D14" s="9">
         <v>20</v>
       </c>
-      <c r="E14" s="24">
+      <c r="E14" s="13">
         <f>IF(B14="",0,6*B14^3+6*B14^2*C14+4*B14*C14^2+2*C14^3)+D14</f>
         <v>354</v>
       </c>
-      <c r="F14" s="20">
+      <c r="F14" s="9">
         <v>1000</v>
       </c>
-      <c r="G14" s="24">
+      <c r="G14" s="13">
         <f>E14*F14*$B$5</f>
         <v>1770000</v>
       </c>
-      <c r="H14" s="25">
+      <c r="H14" s="14">
         <f>$G14/$B$8</f>
         <v>1.77E-2</v>
       </c>
-      <c r="I14" s="25">
+      <c r="I14" s="14">
         <f>$G14/$B$9</f>
         <v>1.0535714285714285E-2</v>
       </c>
-      <c r="J14" s="25">
+      <c r="J14" s="14">
         <f>$G14/$B$10</f>
         <v>3.6874999999999998E-3</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B15" s="23">
+      <c r="B15" s="12">
         <v>9</v>
       </c>
-      <c r="C15" s="23">
+      <c r="C15" s="12">
         <v>6</v>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="9">
         <v>1000</v>
       </c>
-      <c r="E15" s="24">
+      <c r="E15" s="13">
         <f>IF(B15="",0,6*B15^3+6*B15^2*C15+4*B15*C15^2+2*C15^3)+D15</f>
         <v>10018</v>
       </c>
-      <c r="F15" s="20">
+      <c r="F15" s="9">
         <v>500</v>
       </c>
-      <c r="G15" s="24">
+      <c r="G15" s="13">
         <f>E15*F15*$B$5</f>
         <v>25045000</v>
       </c>
-      <c r="H15" s="25">
+      <c r="H15" s="14">
         <f>$G15/$B$8</f>
         <v>0.25045000000000001</v>
       </c>
-      <c r="I15" s="25">
+      <c r="I15" s="14">
         <f>$G15/$B$9</f>
         <v>0.14907738095238096</v>
       </c>
-      <c r="J15" s="25">
+      <c r="J15" s="14">
         <f>$G15/$B$10</f>
         <v>5.2177083333333332E-2</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="20">
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="9">
         <v>2000</v>
       </c>
-      <c r="E16" s="24">
+      <c r="E16" s="13">
         <f>IF(B16="",0,6*B16^3+6*B16^2*C16+4*B16*C16^2+2*C16^3)+D16</f>
         <v>2000</v>
       </c>
-      <c r="F16" s="20">
+      <c r="F16" s="9">
         <v>100</v>
       </c>
-      <c r="G16" s="24">
+      <c r="G16" s="13">
         <f>E16*F16*$B$5</f>
         <v>1000000</v>
       </c>
-      <c r="H16" s="25">
+      <c r="H16" s="14">
         <f>$G16/$B$8</f>
         <v>0.01</v>
       </c>
-      <c r="I16" s="25">
+      <c r="I16" s="14">
         <f>$G16/$B$9</f>
         <v>5.9523809523809521E-3</v>
       </c>
-      <c r="J16" s="25">
+      <c r="J16" s="14">
         <f>$G16/$B$10</f>
         <v>2.0833333333333333E-3</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="24">
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="13">
         <f>$B$6</f>
         <v>20000000</v>
       </c>
-      <c r="H17" s="25">
+      <c r="H17" s="14">
         <f>$G17/$B$8</f>
         <v>0.2</v>
       </c>
-      <c r="I17" s="25">
+      <c r="I17" s="14">
         <f>$G17/$B$9</f>
         <v>0.11904761904761904</v>
       </c>
-      <c r="J17" s="25">
+      <c r="J17" s="14">
         <f>$G17/$B$10</f>
         <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" s="26" t="s">
+      <c r="A18" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="B18" s="27"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="28">
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="17">
         <f>SUM(G14:G17)</f>
         <v>47815000</v>
       </c>
-      <c r="H18" s="29">
+      <c r="H18" s="18">
         <f>SUM(H14:H17)</f>
         <v>0.47815000000000002</v>
       </c>
-      <c r="I18" s="29">
+      <c r="I18" s="18">
         <f>SUM(I14:I17)</f>
         <v>0.28461309523809525</v>
       </c>
-      <c r="J18" s="29">
+      <c r="J18" s="18">
         <f>SUM(J14:J17)</f>
         <v>9.9614583333333326E-2</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="14" t="str">
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="3" t="str">
         <f>IF(H18&lt;=1-$B$7,"Sí","No")</f>
         <v>Sí</v>
       </c>
-      <c r="I19" s="14" t="str">
+      <c r="I19" s="3" t="str">
         <f>IF(I18&lt;=1-$B$7,"Sí","No")</f>
         <v>Sí</v>
       </c>
-      <c r="J19" s="14" t="str">
+      <c r="J19" s="3" t="str">
         <f>IF(J18&lt;=1-$B$7,"Sí","No")</f>
         <v>Sí</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="23"/>
     </row>
     <row r="22" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
     </row>
     <row r="23" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="21"/>
     </row>
     <row r="24" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="21"/>
     </row>
     <row r="25" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="21"/>
     </row>
     <row r="26" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="21"/>
+      <c r="J26" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="A26:J26"/>
-    <mergeCell ref="A21:J21"/>
-    <mergeCell ref="A22:J22"/>
-    <mergeCell ref="A23:J23"/>
     <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="C5:J5"/>
     <mergeCell ref="A25:J25"/>
-    <mergeCell ref="C7:J7"/>
     <mergeCell ref="C8:J8"/>
     <mergeCell ref="C9:J9"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A23:J23"/>
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="C6:J6"/>
     <mergeCell ref="C10:J10"/>
+    <mergeCell ref="A21:J21"/>
     <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
     <mergeCell ref="A4:J4"/>
-    <mergeCell ref="C5:J5"/>
-    <mergeCell ref="C6:J6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>